<commit_message>
Further changes to get calculation of times to align with Bizagi times
</commit_message>
<xml_diff>
--- a/Bizagi/process_1_simulation_results.xlsx
+++ b/Bizagi/process_1_simulation_results.xlsx
@@ -526,34 +526,34 @@
         <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>21.25605975</v>
+        <v>15.44060605</v>
       </c>
       <c r="G2" t="n">
-        <v>37.30676246666667</v>
+        <v>35.81448788333333</v>
       </c>
       <c r="H2" t="n">
-        <v>28.3</v>
+        <v>22.44</v>
       </c>
       <c r="I2" t="n">
-        <v>29.43</v>
+        <v>23.13</v>
       </c>
       <c r="J2" t="n">
-        <v>5.3</v>
+        <v>5.69</v>
       </c>
       <c r="K2" t="n">
-        <v>33.81</v>
+        <v>28.62</v>
       </c>
       <c r="L2" t="n">
-        <v>62.97</v>
+        <v>65.54000000000001</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>13.6</v>
+        <v>14.26</v>
       </c>
       <c r="O2" t="n">
-        <v>6.3</v>
+        <v>6.55</v>
       </c>
     </row>
     <row r="3">
@@ -577,22 +577,22 @@
         <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>3.37</v>
+        <v>1.53</v>
       </c>
       <c r="G3" t="n">
-        <v>9.109999999999999</v>
+        <v>8.07</v>
       </c>
       <c r="H3" t="n">
-        <v>6.48</v>
+        <v>3.64</v>
       </c>
       <c r="I3" t="n">
-        <v>6.24</v>
+        <v>3.34</v>
       </c>
       <c r="J3" t="n">
-        <v>1.61</v>
+        <v>2.04</v>
       </c>
       <c r="K3" t="n">
-        <v>8.44</v>
+        <v>6.72</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -628,34 +628,34 @@
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="G4" t="n">
-        <v>1.79</v>
+        <v>1.98</v>
       </c>
       <c r="H4" t="n">
-        <v>1.11</v>
+        <v>1.21</v>
       </c>
       <c r="I4" t="n">
-        <v>1.18</v>
+        <v>0.97</v>
       </c>
       <c r="J4" t="n">
-        <v>0.35</v>
+        <v>0.54</v>
       </c>
       <c r="K4" t="n">
-        <v>1.46</v>
+        <v>1.95</v>
       </c>
       <c r="L4" t="n">
-        <v>2.89</v>
+        <v>7.52</v>
       </c>
       <c r="M4" t="n">
-        <v>1.05</v>
+        <v>1.12</v>
       </c>
       <c r="N4" t="n">
-        <v>1.84</v>
+        <v>1.94</v>
       </c>
       <c r="O4" t="n">
-        <v>1.44</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="5">
@@ -679,22 +679,22 @@
         <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>3.79</v>
+        <v>3.01</v>
       </c>
       <c r="G5" t="n">
-        <v>7.75</v>
+        <v>6.66</v>
       </c>
       <c r="H5" t="n">
-        <v>5.86</v>
+        <v>3.98</v>
       </c>
       <c r="I5" t="n">
-        <v>5.8</v>
+        <v>3.83</v>
       </c>
       <c r="J5" t="n">
-        <v>1.44</v>
+        <v>0.97</v>
       </c>
       <c r="K5" t="n">
-        <v>7.67</v>
+        <v>4.45</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -730,34 +730,34 @@
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>2.88</v>
+        <v>2.1</v>
       </c>
       <c r="G6" t="n">
-        <v>4.97</v>
+        <v>5.66</v>
       </c>
       <c r="H6" t="n">
-        <v>3.95</v>
+        <v>3.33</v>
       </c>
       <c r="I6" t="n">
-        <v>4.25</v>
+        <v>3.17</v>
       </c>
       <c r="J6" t="n">
-        <v>0.68</v>
+        <v>0.9</v>
       </c>
       <c r="K6" t="n">
-        <v>4.8</v>
+        <v>4.15</v>
       </c>
       <c r="L6" t="n">
-        <v>60.08</v>
+        <v>58.02</v>
       </c>
       <c r="M6" t="n">
-        <v>2.72</v>
+        <v>1.18</v>
       </c>
       <c r="N6" t="n">
-        <v>13.6</v>
+        <v>14.26</v>
       </c>
       <c r="O6" t="n">
-        <v>6.68</v>
+        <v>7.25</v>
       </c>
     </row>
     <row r="7">
@@ -781,22 +781,22 @@
         <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>3.32</v>
+        <v>1.01</v>
       </c>
       <c r="G7" t="n">
-        <v>8.470000000000001</v>
+        <v>8.49</v>
       </c>
       <c r="H7" t="n">
-        <v>4.6</v>
+        <v>3.73</v>
       </c>
       <c r="I7" t="n">
-        <v>4.14</v>
+        <v>3.41</v>
       </c>
       <c r="J7" t="n">
-        <v>1.53</v>
+        <v>2.04</v>
       </c>
       <c r="K7" t="n">
-        <v>6.27</v>
+        <v>6.05</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>

</xml_diff>